<commit_message>
fix(analytics): implement fractional hour interpolation to prevent artificial pacing drops on half-hour cuts
</commit_message>
<xml_diff>
--- a/data/Top_50_Detratores_Canais_Digitais.xlsx
+++ b/data/Top_50_Detratores_Canais_Digitais.xlsx
@@ -821,13 +821,13 @@
         <v>3620.78</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>21627.68</v>
+        <v>20992.84</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>-18006.9</v>
+        <v>-17372.06</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>-0.833</v>
+        <v>-0.828</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>600869</v>
@@ -888,13 +888,13 @@
         <v>1961.14</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>14430.35</v>
+        <v>14006.77</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>-12469.21</v>
+        <v>-12045.63</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>-0.8640000000000001</v>
+        <v>-0.86</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>324969</v>
@@ -945,13 +945,13 @@
         <v>1564.54</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>12556.52</v>
+        <v>12187.94</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-10991.98</v>
+        <v>-10623.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-0.875</v>
+        <v>-0.872</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>510877</v>
@@ -1002,13 +1002,13 @@
         <v>1099</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>10712.65</v>
+        <v>10398.2</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>-9613.65</v>
+        <v>-9299.200000000001</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>-0.897</v>
+        <v>-0.894</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>4436</v>
@@ -1069,13 +1069,13 @@
         <v>1047.42</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>5688.45</v>
+        <v>5521.47</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-4641.03</v>
+        <v>-4474.05</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>-0.8159999999999999</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>47906</v>
@@ -1126,13 +1126,13 @@
         <v>1509.91</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>6128.64</v>
+        <v>5948.75</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>-4618.73</v>
+        <v>-4438.84</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>-0.754</v>
+        <v>-0.746</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>113479</v>
@@ -1183,13 +1183,13 @@
         <v>1730.92</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>6269.46</v>
+        <v>6085.43</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-4538.54</v>
+        <v>-4354.51</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>-0.7240000000000001</v>
+        <v>-0.716</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>99015</v>
@@ -1240,13 +1240,13 @@
         <v>1265.34</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>4553.26</v>
+        <v>4419.61</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>-3287.92</v>
+        <v>-3154.27</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-0.722</v>
+        <v>-0.7140000000000001</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>250037</v>
@@ -1307,13 +1307,13 @@
         <v>6444.5</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>9726.610000000001</v>
+        <v>9441.110000000001</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-3282.11</v>
+        <v>-2996.61</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>-0.337</v>
+        <v>-0.317</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>2104969</v>
@@ -1374,13 +1374,13 @@
         <v>999</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>3771.18</v>
+        <v>3660.48</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>-2772.18</v>
+        <v>-2661.48</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>-0.735</v>
+        <v>-0.727</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>2591</v>
@@ -1441,10 +1441,10 @@
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2397.27</v>
+        <v>2326.9</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-2397.27</v>
+        <v>-2326.9</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>-1</v>
@@ -1508,10 +1508,10 @@
         <v>0</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>2066.49</v>
+        <v>2005.83</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>-2066.49</v>
+        <v>-2005.83</v>
       </c>
       <c r="G16" s="20" t="n">
         <v>-1</v>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1795.93</v>
+        <v>1743.21</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-1795.93</v>
+        <v>-1743.21</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>-1</v>
@@ -1622,13 +1622,13 @@
         <v>260.53</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>1667.57</v>
+        <v>1618.62</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>-1407.04</v>
+        <v>-1358.09</v>
       </c>
       <c r="G18" s="20" t="n">
-        <v>-0.8440000000000001</v>
+        <v>-0.8390000000000001</v>
       </c>
       <c r="H18" s="21" t="n">
         <v>70898</v>
@@ -1677,39 +1677,39 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>10050648</t>
+          <t>10030120</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
+          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>4632</v>
+        <v>0</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>6017.89</v>
+        <v>1254.19</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-1385.89</v>
+        <v>-1254.19</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.23</v>
+        <v>-1</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>52129</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>41.41</v>
+        <v>1252</v>
+      </c>
+      <c r="I19" s="33" t="n">
+        <v>0.99</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K19" s="7" t="n">
-        <v>988.22</v>
+        <v>1301.17</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="M19" s="7" t="n">
-        <v>988.22</v>
+        <v>1301.17</v>
       </c>
       <c r="N19" s="13" t="n">
         <v>0</v>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="Q19" s="14" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -1744,39 +1744,39 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>100000855</t>
+          <t>10020597</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>OLEO CAB ELSEVE 100ML EXTRAORDINARIO</t>
+          <t>TOALHAS UMED PAMPERS LV4 PG3 ALOE VERA</t>
         </is>
       </c>
       <c r="D20" s="18" t="n">
-        <v>1199.73</v>
+        <v>837</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>2497.77</v>
+        <v>2067.17</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>-1298.04</v>
+        <v>-1230.17</v>
       </c>
       <c r="G20" s="20" t="n">
-        <v>-0.52</v>
+        <v>-0.595</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>119320</v>
+        <v>97029</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>94.77</v>
+        <v>77.06999999999999</v>
       </c>
       <c r="J20" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K20" s="18" t="n">
-        <v>39.99</v>
+        <v>35.9</v>
       </c>
       <c r="L20" s="24" t="inlineStr">
         <is>
@@ -1784,14 +1784,14 @@
         </is>
       </c>
       <c r="M20" s="18" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="N20" s="30" t="n">
-        <v>0.294</v>
+        <v>36.89</v>
+      </c>
+      <c r="N20" s="29" t="n">
+        <v>-0.027</v>
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P20" s="24" t="inlineStr">
@@ -1799,9 +1799,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q20" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 30.90)</t>
+      <c r="Q20" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1811,39 +1811,39 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>10020597</t>
+          <t>100000855</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>TOALHAS UMED PAMPERS LV4 PG3 ALOE VERA</t>
+          <t>OLEO CAB ELSEVE 100ML EXTRAORDINARIO</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>837</v>
+        <v>1199.73</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>2129.69</v>
+        <v>2424.46</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-1292.69</v>
+        <v>-1224.73</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>-0.607</v>
+        <v>-0.505</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>97029</v>
+        <v>119320</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>77.06999999999999</v>
+        <v>94.77</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K21" s="7" t="n">
-        <v>35.9</v>
+        <v>39.99</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
@@ -1851,14 +1851,14 @@
         </is>
       </c>
       <c r="M21" s="7" t="n">
-        <v>36.89</v>
-      </c>
-      <c r="N21" s="13" t="n">
-        <v>-0.027</v>
+        <v>30.9</v>
+      </c>
+      <c r="N21" s="31" t="n">
+        <v>0.294</v>
       </c>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P21" s="12" t="inlineStr">
@@ -1866,9 +1866,9 @@
           <t>Detrator Moderado</t>
         </is>
       </c>
-      <c r="Q21" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q21" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 30.90)</t>
         </is>
       </c>
     </row>
@@ -1878,39 +1878,39 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>10030120</t>
+          <t>10050648</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>RYBELSUS 7MG 30CP NOVO NORDISK</t>
+          <t>POVIZTRA 1MG 3ML EUROFARMA</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>0</v>
+        <v>4632</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>1292.12</v>
+        <v>5841.24</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>-1292.12</v>
+        <v>-1209.24</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>-1</v>
+        <v>-0.207</v>
       </c>
       <c r="H22" s="21" t="n">
-        <v>1252</v>
-      </c>
-      <c r="I22" s="32" t="n">
-        <v>0.99</v>
+        <v>52129</v>
+      </c>
+      <c r="I22" s="22" t="n">
+        <v>41.41</v>
       </c>
       <c r="J22" s="15" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K22" s="18" t="n">
-        <v>1301.17</v>
+        <v>988.22</v>
       </c>
       <c r="L22" s="24" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="M22" s="18" t="n">
-        <v>1301.17</v>
+        <v>988.22</v>
       </c>
       <c r="N22" s="29" t="n">
         <v>0</v>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="Q22" s="26" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -1957,13 +1957,13 @@
         <v>665.1</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>1906.87</v>
+        <v>1850.89</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-1241.77</v>
+        <v>-1185.79</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>-0.6509999999999999</v>
+        <v>-0.6409999999999999</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>40006</v>
@@ -2002,40 +2002,46 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>10052539</t>
+          <t>10025098</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
+          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
         </is>
       </c>
       <c r="D24" s="18" t="n">
-        <v>629.5</v>
+        <v>0</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>1801.21</v>
+        <v>1135.4</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>-1171.71</v>
+        <v>-1135.4</v>
       </c>
       <c r="G24" s="20" t="n">
-        <v>-0.6509999999999999</v>
+        <v>-1</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>16483</v>
-      </c>
-      <c r="I24" s="22" t="n">
-        <v>13.09</v>
+        <v>227</v>
+      </c>
+      <c r="I24" s="32" t="n">
+        <v>0.18</v>
       </c>
       <c r="J24" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr"/>
-      <c r="M24" s="23" t="inlineStr"/>
+      <c r="L24" s="24" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M24" s="18" t="n">
+        <v>1212.9</v>
+      </c>
       <c r="N24" s="25" t="inlineStr"/>
       <c r="O24" s="24" t="inlineStr">
         <is>
@@ -2049,7 +2055,7 @@
       </c>
       <c r="Q24" s="26" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2059,46 +2065,40 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>10025098</t>
+          <t>10052539</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>AJOVY 225MG 1,5ML SER PREENC TEVA</t>
+          <t>FR PAMPERS PANTS AJUSTE TOTAL MAX XG 82U</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>0</v>
+        <v>629.5</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>1169.74</v>
+        <v>1748.34</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-1169.74</v>
+        <v>-1118.84</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>-1</v>
+        <v>-0.64</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>227</v>
-      </c>
-      <c r="I25" s="33" t="n">
-        <v>0.18</v>
+        <v>16483</v>
+      </c>
+      <c r="I25" s="11" t="n">
+        <v>13.09</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K25" s="27" t="inlineStr"/>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M25" s="7" t="n">
-        <v>1212.9</v>
-      </c>
+      <c r="L25" s="12" t="inlineStr"/>
+      <c r="M25" s="27" t="inlineStr"/>
       <c r="N25" s="28" t="inlineStr"/>
       <c r="O25" s="12" t="inlineStr">
         <is>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="Q25" s="14" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2134,13 +2134,13 @@
         <v>137.31</v>
       </c>
       <c r="E26" s="18" t="n">
-        <v>1205.34</v>
+        <v>1169.96</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>-1068.03</v>
+        <v>-1032.65</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>-0.8859999999999999</v>
+        <v>-0.883</v>
       </c>
       <c r="H26" s="21" t="n">
         <v>32286</v>
@@ -2201,13 +2201,13 @@
         <v>455</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>1474.18</v>
+        <v>1430.91</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>-1019.18</v>
+        <v>-975.91</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>-0.6909999999999999</v>
+        <v>-0.6820000000000001</v>
       </c>
       <c r="H27" s="10" t="n">
         <v>137002</v>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="P27" s="12" t="inlineStr">
         <is>
-          <t>Detrator Moderado</t>
+          <t>Neutro</t>
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr">
@@ -2256,44 +2256,54 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>10037164</t>
+          <t>10049738</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>TOALHAS UMED PAMPERS CUIDADO DE BEBE C/TAMPA LV4 PG3</t>
+          <t>OLIRE 6MG/ML 3ML 3APLIC INJ EMS</t>
         </is>
       </c>
       <c r="D28" s="18" t="n">
-        <v>563.8200000000001</v>
+        <v>0</v>
       </c>
       <c r="E28" s="18" t="n">
-        <v>1452.3</v>
+        <v>850.25</v>
       </c>
       <c r="F28" s="19" t="n">
-        <v>-888.48</v>
+        <v>-850.25</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>-0.612</v>
+        <v>-1</v>
       </c>
       <c r="H28" s="21" t="n">
-        <v>64320</v>
-      </c>
-      <c r="I28" s="22" t="n">
-        <v>51.09</v>
+        <v>1336</v>
+      </c>
+      <c r="I28" s="32" t="n">
+        <v>1.06</v>
       </c>
       <c r="J28" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr"/>
-      <c r="M28" s="23" t="inlineStr"/>
-      <c r="N28" s="25" t="inlineStr"/>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K28" s="18" t="n">
+        <v>866.24</v>
+      </c>
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>PANVEL</t>
+        </is>
+      </c>
+      <c r="M28" s="18" t="n">
+        <v>866.24</v>
+      </c>
+      <c r="N28" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="O28" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P28" s="24" t="inlineStr">
@@ -2303,7 +2313,7 @@
       </c>
       <c r="Q28" s="26" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2313,54 +2323,44 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>10049738</t>
+          <t>10037164</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>OLIRE 6MG/ML 3ML 3APLIC INJ EMS</t>
+          <t>TOALHAS UMED PAMPERS CUIDADO DE BEBE C/TAMPA LV4 PG3</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>0</v>
+        <v>563.8200000000001</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>875.96</v>
+        <v>1409.67</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-875.96</v>
+        <v>-845.85</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>-1</v>
+        <v>-0.6</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>1336</v>
-      </c>
-      <c r="I29" s="33" t="n">
-        <v>1.06</v>
+        <v>64320</v>
+      </c>
+      <c r="I29" s="11" t="n">
+        <v>51.09</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="n">
-        <v>866.24</v>
-      </c>
-      <c r="L29" s="12" t="inlineStr">
-        <is>
-          <t>PANVEL</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="n">
-        <v>866.24</v>
-      </c>
-      <c r="N29" s="13" t="n">
-        <v>0</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K29" s="27" t="inlineStr"/>
+      <c r="L29" s="12" t="inlineStr"/>
+      <c r="M29" s="27" t="inlineStr"/>
+      <c r="N29" s="28" t="inlineStr"/>
       <c r="O29" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P29" s="12" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="Q29" s="14" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2392,13 +2392,13 @@
         <v>1048.6</v>
       </c>
       <c r="E30" s="18" t="n">
-        <v>1907.91</v>
+        <v>1851.91</v>
       </c>
       <c r="F30" s="19" t="n">
-        <v>-859.3099999999999</v>
+        <v>-803.3099999999999</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>-0.45</v>
+        <v>-0.434</v>
       </c>
       <c r="H30" s="21" t="n">
         <v>27826</v>
@@ -2459,13 +2459,13 @@
         <v>491.16</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>1299.71</v>
+        <v>1261.56</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-808.55</v>
+        <v>-770.4</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>-0.622</v>
+        <v>-0.611</v>
       </c>
       <c r="H31" s="10" t="n">
         <v>4986</v>
@@ -2526,13 +2526,13 @@
         <v>1475.85</v>
       </c>
       <c r="E32" s="18" t="n">
-        <v>2267.75</v>
+        <v>2201.18</v>
       </c>
       <c r="F32" s="19" t="n">
-        <v>-791.9</v>
+        <v>-725.33</v>
       </c>
       <c r="G32" s="20" t="n">
-        <v>-0.349</v>
+        <v>-0.33</v>
       </c>
       <c r="H32" s="21" t="n">
         <v>55490</v>
@@ -2583,13 +2583,13 @@
         <v>286.13</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>1017.58</v>
+        <v>987.72</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-731.45</v>
+        <v>-701.59</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>-0.7190000000000001</v>
+        <v>-0.71</v>
       </c>
       <c r="H33" s="10" t="n">
         <v>282367</v>
@@ -2630,50 +2630,54 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>100014938</t>
+          <t>10037163</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>LA ROCHE CICAPLAST BAUME B5 20ML</t>
+          <t>CANABIDIOL 100MG/ML 30ML EASE LABS (B1)</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
-        <v>796.2</v>
+        <v>0</v>
       </c>
       <c r="E34" s="18" t="n">
-        <v>1470.9</v>
+        <v>647.64</v>
       </c>
       <c r="F34" s="19" t="n">
-        <v>-674.7</v>
+        <v>-647.64</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>-0.459</v>
+        <v>-1</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>100343</v>
-      </c>
-      <c r="I34" s="22" t="n">
-        <v>79.7</v>
+        <v>22</v>
+      </c>
+      <c r="I34" s="32" t="n">
+        <v>0.02</v>
       </c>
       <c r="J34" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr"/>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K34" s="18" t="n">
+        <v>1142</v>
+      </c>
       <c r="L34" s="24" t="inlineStr">
         <is>
-          <t>NISSEI</t>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M34" s="18" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="N34" s="25" t="inlineStr"/>
+        <v>1141.99</v>
+      </c>
+      <c r="N34" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="O34" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P34" s="24" t="inlineStr">
@@ -2683,7 +2687,7 @@
       </c>
       <c r="Q34" s="26" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2693,54 +2697,50 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>10037163</t>
+          <t>100014938</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>CANABIDIOL 100MG/ML 30ML EASE LABS (B1)</t>
+          <t>LA ROCHE CICAPLAST BAUME B5 20ML</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>0</v>
+        <v>796.2</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>667.23</v>
+        <v>1427.72</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>-667.23</v>
+        <v>-631.52</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>-1</v>
+        <v>-0.442</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="I35" s="33" t="n">
-        <v>0.02</v>
+        <v>100343</v>
+      </c>
+      <c r="I35" s="11" t="n">
+        <v>79.7</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
-        </is>
-      </c>
-      <c r="K35" s="7" t="n">
-        <v>1142</v>
-      </c>
+          <t>📉 Demanda Normal</t>
+        </is>
+      </c>
+      <c r="K35" s="27" t="inlineStr"/>
       <c r="L35" s="12" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M35" s="7" t="n">
-        <v>1141.99</v>
-      </c>
-      <c r="N35" s="13" t="n">
-        <v>0</v>
-      </c>
+        <v>39.9</v>
+      </c>
+      <c r="N35" s="28" t="inlineStr"/>
       <c r="O35" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P35" s="12" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="Q35" s="14" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -2760,31 +2760,31 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>10026836</t>
+          <t>10051359</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>IUMI ES 3MG+20MCG 120CP REV LIBBS</t>
+          <t>SENSOR SMART 2.0 GX-01S MEDLEVENSOHN</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
-        <v>1482.3</v>
+        <v>309</v>
       </c>
       <c r="E36" s="18" t="n">
-        <v>2122.46</v>
+        <v>915.23</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>-640.16</v>
+        <v>-606.23</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>-0.302</v>
+        <v>-0.662</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>7710</v>
+        <v>1921</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>6.12</v>
+        <v>1.53</v>
       </c>
       <c r="J36" s="15" t="inlineStr">
         <is>
@@ -2792,18 +2792,18 @@
         </is>
       </c>
       <c r="K36" s="18" t="n">
-        <v>153.23</v>
+        <v>309</v>
       </c>
       <c r="L36" s="24" t="inlineStr">
         <is>
-          <t>DROGARAIA</t>
+          <t>AMAZON</t>
         </is>
       </c>
       <c r="M36" s="18" t="n">
-        <v>173.71</v>
+        <v>449</v>
       </c>
       <c r="N36" s="29" t="n">
-        <v>-0.118</v>
+        <v>-0.312</v>
       </c>
       <c r="O36" s="24" t="inlineStr">
         <is>
@@ -2827,31 +2827,31 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>10051359</t>
+          <t>10041853</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>SENSOR SMART 2.0 GX-01S MEDLEVENSOHN</t>
+          <t>FR PAMPERS PANTS PREMIUM CARE XXG 90UN</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>309</v>
+        <v>692.6</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>942.91</v>
+        <v>1285.71</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-633.91</v>
+        <v>-593.11</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>-0.672</v>
+        <v>-0.461</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1921</v>
+        <v>3127</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>1.53</v>
+        <v>2.48</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -2859,22 +2859,22 @@
         </is>
       </c>
       <c r="K37" s="7" t="n">
-        <v>309</v>
+        <v>169.9</v>
       </c>
       <c r="L37" s="12" t="inlineStr">
         <is>
-          <t>AMAZON</t>
+          <t>PANVEL</t>
         </is>
       </c>
       <c r="M37" s="7" t="n">
-        <v>449</v>
+        <v>169.9</v>
       </c>
       <c r="N37" s="13" t="n">
-        <v>-0.312</v>
+        <v>0</v>
       </c>
       <c r="O37" s="12" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P37" s="12" t="inlineStr">
@@ -2894,54 +2894,50 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>10041853</t>
+          <t>10028253</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>FR PAMPERS PANTS PREMIUM CARE XXG 90UN</t>
+          <t>COGLIVE 24MG 60CAP DURA LIB PROL LIBBS (C1)</t>
         </is>
       </c>
       <c r="D38" s="18" t="n">
-        <v>692.6</v>
+        <v>0</v>
       </c>
       <c r="E38" s="18" t="n">
-        <v>1324.59</v>
+        <v>580.84</v>
       </c>
       <c r="F38" s="19" t="n">
-        <v>-631.99</v>
+        <v>-580.84</v>
       </c>
       <c r="G38" s="20" t="n">
-        <v>-0.477</v>
+        <v>-1</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>3127</v>
-      </c>
-      <c r="I38" s="22" t="n">
-        <v>2.48</v>
+        <v>1575</v>
+      </c>
+      <c r="I38" s="32" t="n">
+        <v>1.25</v>
       </c>
       <c r="J38" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K38" s="18" t="n">
-        <v>169.9</v>
-      </c>
+          <t>🚨 Ruptura Logística</t>
+        </is>
+      </c>
+      <c r="K38" s="23" t="inlineStr"/>
       <c r="L38" s="24" t="inlineStr">
         <is>
-          <t>PANVEL</t>
+          <t>NISSEI</t>
         </is>
       </c>
       <c r="M38" s="18" t="n">
-        <v>169.9</v>
-      </c>
-      <c r="N38" s="29" t="n">
-        <v>0</v>
-      </c>
+        <v>388.97</v>
+      </c>
+      <c r="N38" s="25" t="inlineStr"/>
       <c r="O38" s="24" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P38" s="24" t="inlineStr">
@@ -2951,7 +2947,7 @@
       </c>
       <c r="Q38" s="26" t="inlineStr">
         <is>
-          <t>Ação Promocional / Destaque Home</t>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -2961,54 +2957,54 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>10046027</t>
+          <t>10026836</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>FR PAMPERS SUPERSEC XG 56UN</t>
+          <t>IUMI ES 3MG+20MCG 120CP REV LIBBS</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>2309.55</v>
+        <v>1482.3</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>2911.17</v>
+        <v>2060.16</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-601.62</v>
+        <v>-577.86</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>-0.207</v>
+        <v>-0.28</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>62068</v>
+        <v>7710</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>49.3</v>
+        <v>6.12</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K39" s="7" t="n">
-        <v>85.90000000000001</v>
+        <v>153.23</v>
       </c>
       <c r="L39" s="12" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>DROGARAIA</t>
         </is>
       </c>
       <c r="M39" s="7" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="N39" s="31" t="n">
-        <v>0.434</v>
+        <v>173.71</v>
+      </c>
+      <c r="N39" s="13" t="n">
+        <v>-0.118</v>
       </c>
       <c r="O39" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P39" s="12" t="inlineStr">
@@ -3016,9 +3012,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q39" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Precopopular R$ 59.90)</t>
+      <c r="Q39" s="14" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3028,31 +3024,31 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>10032148</t>
+          <t>10006909</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>APTAMIL PROFUTURA GOLD 1 800G DANONE</t>
+          <t>OSCAL D 500MG+1000UI 60CP REV OPELLA</t>
         </is>
       </c>
       <c r="D40" s="18" t="n">
-        <v>372.97</v>
+        <v>0</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>973.9</v>
+        <v>574.61</v>
       </c>
       <c r="F40" s="19" t="n">
-        <v>-600.9299999999999</v>
+        <v>-574.61</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>-0.617</v>
+        <v>-1</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>24608</v>
+        <v>3164</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>19.55</v>
+        <v>2.51</v>
       </c>
       <c r="J40" s="15" t="inlineStr">
         <is>
@@ -3060,7 +3056,7 @@
         </is>
       </c>
       <c r="K40" s="18" t="n">
-        <v>130.99</v>
+        <v>166.64</v>
       </c>
       <c r="L40" s="24" t="inlineStr">
         <is>
@@ -3068,10 +3064,10 @@
         </is>
       </c>
       <c r="M40" s="18" t="n">
-        <v>119.59</v>
+        <v>150.99</v>
       </c>
       <c r="N40" s="30" t="n">
-        <v>0.095</v>
+        <v>0.104</v>
       </c>
       <c r="O40" s="24" t="inlineStr">
         <is>
@@ -3085,7 +3081,7 @@
       </c>
       <c r="Q40" s="17" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Amazon R$ 119.59)</t>
+          <t>Reprecificar no Digital (Amazon R$ 150.99)</t>
         </is>
       </c>
     </row>
@@ -3095,46 +3091,40 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>10028253</t>
+          <t>10001098</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>COGLIVE 24MG 60CAP DURA LIB PROL LIBBS (C1)</t>
+          <t>TOALHAS UMED HUGGIES 192UN HIDRATACAO</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>0</v>
+        <v>161.97</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>598.41</v>
+        <v>735.02</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-598.41</v>
+        <v>-573.05</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>-1</v>
+        <v>-0.78</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>1575</v>
-      </c>
-      <c r="I41" s="33" t="n">
-        <v>1.25</v>
+        <v>65288</v>
+      </c>
+      <c r="I41" s="11" t="n">
+        <v>51.86</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K41" s="27" t="inlineStr"/>
-      <c r="L41" s="12" t="inlineStr">
-        <is>
-          <t>NISSEI</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="n">
-        <v>388.97</v>
-      </c>
+      <c r="L41" s="12" t="inlineStr"/>
+      <c r="M41" s="27" t="inlineStr"/>
       <c r="N41" s="28" t="inlineStr"/>
       <c r="O41" s="12" t="inlineStr">
         <is>
@@ -3148,7 +3138,7 @@
       </c>
       <c r="Q41" s="14" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3158,44 +3148,54 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>10001098</t>
+          <t>10032148</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>TOALHAS UMED HUGGIES 192UN HIDRATACAO</t>
+          <t>APTAMIL PROFUTURA GOLD 1 800G DANONE</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
-        <v>161.97</v>
+        <v>372.97</v>
       </c>
       <c r="E42" s="18" t="n">
-        <v>757.25</v>
+        <v>945.3099999999999</v>
       </c>
       <c r="F42" s="19" t="n">
-        <v>-595.28</v>
+        <v>-572.34</v>
       </c>
       <c r="G42" s="20" t="n">
-        <v>-0.7859999999999999</v>
+        <v>-0.605</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>65288</v>
+        <v>24608</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>51.86</v>
+        <v>19.55</v>
       </c>
       <c r="J42" s="15" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr"/>
-      <c r="L42" s="24" t="inlineStr"/>
-      <c r="M42" s="23" t="inlineStr"/>
-      <c r="N42" s="25" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K42" s="18" t="n">
+        <v>130.99</v>
+      </c>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>AMAZON</t>
+        </is>
+      </c>
+      <c r="M42" s="18" t="n">
+        <v>119.59</v>
+      </c>
+      <c r="N42" s="30" t="n">
+        <v>0.095</v>
+      </c>
       <c r="O42" s="24" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P42" s="24" t="inlineStr">
@@ -3203,9 +3203,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q42" s="26" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q42" s="17" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Amazon R$ 119.59)</t>
         </is>
       </c>
     </row>
@@ -3215,54 +3215,54 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>10006909</t>
+          <t>10050639</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>OSCAL D 500MG+1000UI 60CP REV OPELLA</t>
+          <t>EXTENSIOR 0,25MG+0,5MG 1,5ML NOVO EUROFARMA</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>591.98</v>
+        <v>542.25</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-591.98</v>
+        <v>-542.25</v>
       </c>
       <c r="G43" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>3164</v>
-      </c>
-      <c r="I43" s="11" t="n">
-        <v>2.51</v>
+        <v>599</v>
+      </c>
+      <c r="I43" s="33" t="n">
+        <v>0.48</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>🚨 Ruptura Logística</t>
         </is>
       </c>
       <c r="K43" s="7" t="n">
-        <v>166.64</v>
+        <v>955.85</v>
       </c>
       <c r="L43" s="12" t="inlineStr">
         <is>
-          <t>AMAZON</t>
+          <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M43" s="7" t="n">
-        <v>150.99</v>
-      </c>
-      <c r="N43" s="31" t="n">
-        <v>0.104</v>
+        <v>955.85</v>
+      </c>
+      <c r="N43" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="O43" s="12" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P43" s="12" t="inlineStr">
@@ -3270,9 +3270,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q43" s="6" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 150.99)</t>
+      <c r="Q43" s="14" t="inlineStr">
+        <is>
+          <t>Abastecimento Emergencial Lojas/CD</t>
         </is>
       </c>
     </row>
@@ -3282,31 +3282,31 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>10026927</t>
+          <t>10100057</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>NANLAC SUPREME 800G NESTLE</t>
+          <t>PREGOMIN PEPTI 400G DANONE</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>759.4299999999999</v>
+        <v>0</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>1322.86</v>
+        <v>540.03</v>
       </c>
       <c r="F44" s="19" t="n">
-        <v>-563.4299999999999</v>
+        <v>-540.03</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>-0.426</v>
+        <v>-1</v>
       </c>
       <c r="H44" s="21" t="n">
-        <v>32374</v>
+        <v>4098</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>25.71</v>
+        <v>3.25</v>
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
@@ -3314,18 +3314,18 @@
         </is>
       </c>
       <c r="K44" s="18" t="n">
-        <v>108.49</v>
+        <v>261.99</v>
       </c>
       <c r="L44" s="24" t="inlineStr">
         <is>
-          <t>PREÇO POPULAR</t>
+          <t>AMAZON</t>
         </is>
       </c>
       <c r="M44" s="18" t="n">
-        <v>97.69</v>
+        <v>164.9</v>
       </c>
       <c r="N44" s="30" t="n">
-        <v>0.111</v>
+        <v>0.589</v>
       </c>
       <c r="O44" s="24" t="inlineStr">
         <is>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="Q44" s="17" t="inlineStr">
         <is>
-          <t>Reprecificar no Digital (Precopopular R$ 97.69)</t>
+          <t>Reprecificar no Digital (Amazon R$ 164.90)</t>
         </is>
       </c>
     </row>
@@ -3349,39 +3349,39 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>10050639</t>
+          <t>100020823</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>EXTENSIOR 0,25MG+0,5MG 1,5ML NOVO EUROFARMA</t>
+          <t>VICK XPE 44E 120ML PROCTER</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>0</v>
+        <v>89.36</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>558.64</v>
+        <v>620.72</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-558.64</v>
+        <v>-531.36</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>-1</v>
+        <v>-0.856</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>599</v>
-      </c>
-      <c r="I45" s="33" t="n">
-        <v>0.48</v>
+        <v>95247</v>
+      </c>
+      <c r="I45" s="11" t="n">
+        <v>75.65000000000001</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>🚨 Ruptura Logística</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K45" s="7" t="n">
-        <v>955.85</v>
+        <v>35.74</v>
       </c>
       <c r="L45" s="12" t="inlineStr">
         <is>
@@ -3389,14 +3389,14 @@
         </is>
       </c>
       <c r="M45" s="7" t="n">
-        <v>955.85</v>
+        <v>36.34</v>
       </c>
       <c r="N45" s="13" t="n">
-        <v>0</v>
+        <v>-0.017</v>
       </c>
       <c r="O45" s="12" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Líder de Preço</t>
         </is>
       </c>
       <c r="P45" s="12" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="Q45" s="14" t="inlineStr">
         <is>
-          <t>Abastecimento Emergencial Lojas/CD</t>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3416,54 +3416,54 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>10100057</t>
+          <t>10040753</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>PREGOMIN PEPTI 400G DANONE</t>
+          <t>LYBERDIA 30MG 30CAPS EMS (A3)</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>556.36</v>
+        <v>528.7</v>
       </c>
       <c r="F46" s="19" t="n">
-        <v>-556.36</v>
+        <v>-528.7</v>
       </c>
       <c r="G46" s="20" t="n">
         <v>-1</v>
       </c>
       <c r="H46" s="21" t="n">
-        <v>4098</v>
+        <v>3124</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>3.25</v>
+        <v>2.48</v>
       </c>
       <c r="J46" s="15" t="inlineStr">
         <is>
-          <t>🏷️ Preço Desalinhado</t>
+          <t>📉 Demanda Normal</t>
         </is>
       </c>
       <c r="K46" s="18" t="n">
-        <v>261.99</v>
+        <v>367.27</v>
       </c>
       <c r="L46" s="24" t="inlineStr">
         <is>
-          <t>AMAZON</t>
+          <t>PREÇO POPULAR</t>
         </is>
       </c>
       <c r="M46" s="18" t="n">
-        <v>164.9</v>
-      </c>
-      <c r="N46" s="30" t="n">
-        <v>0.589</v>
+        <v>367.27</v>
+      </c>
+      <c r="N46" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="O46" s="24" t="inlineStr">
         <is>
-          <t>São João Mais Cara</t>
+          <t>Preço Alinhado</t>
         </is>
       </c>
       <c r="P46" s="24" t="inlineStr">
@@ -3471,9 +3471,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q46" s="17" t="inlineStr">
-        <is>
-          <t>Reprecificar no Digital (Amazon R$ 164.90)</t>
+      <c r="Q46" s="26" t="inlineStr">
+        <is>
+          <t>Ação Promocional / Destaque Home</t>
         </is>
       </c>
     </row>
@@ -3483,39 +3483,39 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>100020823</t>
+          <t>10026927</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>VICK XPE 44E 120ML PROCTER</t>
+          <t>NANLAC SUPREME 800G NESTLE</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>89.36</v>
+        <v>759.4299999999999</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>639.49</v>
+        <v>1284.03</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-550.13</v>
+        <v>-524.6</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>-0.86</v>
+        <v>-0.409</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>95247</v>
+        <v>32374</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>75.65000000000001</v>
+        <v>25.71</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
+          <t>🏷️ Preço Desalinhado</t>
         </is>
       </c>
       <c r="K47" s="7" t="n">
-        <v>35.74</v>
+        <v>108.49</v>
       </c>
       <c r="L47" s="12" t="inlineStr">
         <is>
@@ -3523,14 +3523,14 @@
         </is>
       </c>
       <c r="M47" s="7" t="n">
-        <v>36.34</v>
-      </c>
-      <c r="N47" s="13" t="n">
-        <v>-0.017</v>
+        <v>97.69</v>
+      </c>
+      <c r="N47" s="31" t="n">
+        <v>0.111</v>
       </c>
       <c r="O47" s="12" t="inlineStr">
         <is>
-          <t>Líder de Preço</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P47" s="12" t="inlineStr">
@@ -3538,9 +3538,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q47" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q47" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 97.69)</t>
         </is>
       </c>
     </row>
@@ -3550,54 +3550,44 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>10040753</t>
+          <t>100008756</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>LYBERDIA 30MG 30CAPS EMS (A3)</t>
+          <t>LEITE NEOCATE LCP 400G DANONE</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
-        <v>0</v>
+        <v>299.16</v>
       </c>
       <c r="E48" s="18" t="n">
-        <v>544.6900000000001</v>
+        <v>816.61</v>
       </c>
       <c r="F48" s="19" t="n">
-        <v>-544.6900000000001</v>
+        <v>-517.45</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>-1</v>
+        <v>-0.634</v>
       </c>
       <c r="H48" s="21" t="n">
-        <v>3124</v>
+        <v>3000</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>2.48</v>
+        <v>2.38</v>
       </c>
       <c r="J48" s="15" t="inlineStr">
         <is>
           <t>📉 Demanda Normal</t>
         </is>
       </c>
-      <c r="K48" s="18" t="n">
-        <v>367.27</v>
-      </c>
-      <c r="L48" s="24" t="inlineStr">
-        <is>
-          <t>PREÇO POPULAR</t>
-        </is>
-      </c>
-      <c r="M48" s="18" t="n">
-        <v>367.27</v>
-      </c>
-      <c r="N48" s="29" t="n">
-        <v>0</v>
-      </c>
+      <c r="K48" s="23" t="inlineStr"/>
+      <c r="L48" s="24" t="inlineStr"/>
+      <c r="M48" s="23" t="inlineStr"/>
+      <c r="N48" s="25" t="inlineStr"/>
       <c r="O48" s="24" t="inlineStr">
         <is>
-          <t>Preço Alinhado</t>
+          <t>Não Monitorado</t>
         </is>
       </c>
       <c r="P48" s="24" t="inlineStr">
@@ -3617,44 +3607,54 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>100008756</t>
+          <t>10046027</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>LEITE NEOCATE LCP 400G DANONE</t>
+          <t>FR PAMPERS SUPERSEC XG 56UN</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>299.16</v>
+        <v>2309.55</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>841.3099999999999</v>
+        <v>2825.72</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-542.15</v>
+        <v>-516.17</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>-0.644</v>
+        <v>-0.183</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>3000</v>
+        <v>62068</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>2.38</v>
+        <v>49.3</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>📉 Demanda Normal</t>
-        </is>
-      </c>
-      <c r="K49" s="27" t="inlineStr"/>
-      <c r="L49" s="12" t="inlineStr"/>
-      <c r="M49" s="27" t="inlineStr"/>
-      <c r="N49" s="28" t="inlineStr"/>
+          <t>🏷️ Preço Desalinhado</t>
+        </is>
+      </c>
+      <c r="K49" s="7" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="L49" s="12" t="inlineStr">
+        <is>
+          <t>PREÇO POPULAR</t>
+        </is>
+      </c>
+      <c r="M49" s="7" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="N49" s="31" t="n">
+        <v>0.434</v>
+      </c>
       <c r="O49" s="12" t="inlineStr">
         <is>
-          <t>Não Monitorado</t>
+          <t>São João Mais Cara</t>
         </is>
       </c>
       <c r="P49" s="12" t="inlineStr">
@@ -3662,9 +3662,9 @@
           <t>Neutro</t>
         </is>
       </c>
-      <c r="Q49" s="14" t="inlineStr">
-        <is>
-          <t>Ação Promocional / Destaque Home</t>
+      <c r="Q49" s="6" t="inlineStr">
+        <is>
+          <t>Reprecificar no Digital (Precopopular R$ 59.90)</t>
         </is>
       </c>
     </row>
@@ -3686,13 +3686,13 @@
         <v>239.8</v>
       </c>
       <c r="E50" s="18" t="n">
-        <v>767.8</v>
+        <v>745.27</v>
       </c>
       <c r="F50" s="19" t="n">
-        <v>-528</v>
+        <v>-505.47</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>-0.6879999999999999</v>
+        <v>-0.6779999999999999</v>
       </c>
       <c r="H50" s="21" t="n">
         <v>31768</v>
@@ -3743,10 +3743,10 @@
         <v>0</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>520.74</v>
+        <v>505.46</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-520.74</v>
+        <v>-505.46</v>
       </c>
       <c r="G51" s="9" t="n">
         <v>-1</v>
@@ -3810,10 +3810,10 @@
         <v>0</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>497.75</v>
+        <v>483.13</v>
       </c>
       <c r="F52" s="19" t="n">
-        <v>-497.75</v>
+        <v>-483.13</v>
       </c>
       <c r="G52" s="20" t="n">
         <v>-1</v>
@@ -3865,31 +3865,31 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>10041262</t>
+          <t>10041263</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX XG 80</t>
+          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>1562.09</v>
+        <v>143.99</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>2033.47</v>
+        <v>593.3</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-471.38</v>
+        <v>-449.31</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>-0.232</v>
+        <v>-0.757</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>6935</v>
+        <v>3937</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>5.51</v>
+        <v>3.13</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
@@ -3922,31 +3922,31 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>10041263</t>
+          <t>100007100</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>FR HUGGIES ROUPINHA ACOLCHOADA MAX G 88U</t>
+          <t>QUETIAPINA 25MG 30CP REV GEN EMS (C1)</t>
         </is>
       </c>
       <c r="D54" s="18" t="n">
-        <v>143.99</v>
+        <v>138.72</v>
       </c>
       <c r="E54" s="18" t="n">
-        <v>611.24</v>
+        <v>567.84</v>
       </c>
       <c r="F54" s="19" t="n">
-        <v>-467.25</v>
+        <v>-429.12</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>-0.764</v>
+        <v>-0.7559999999999999</v>
       </c>
       <c r="H54" s="21" t="n">
-        <v>3937</v>
+        <v>131530</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>3.13</v>
+        <v>104.47</v>
       </c>
       <c r="J54" s="15" t="inlineStr">
         <is>
@@ -3954,8 +3954,14 @@
         </is>
       </c>
       <c r="K54" s="23" t="inlineStr"/>
-      <c r="L54" s="24" t="inlineStr"/>
-      <c r="M54" s="23" t="inlineStr"/>
+      <c r="L54" s="24" t="inlineStr">
+        <is>
+          <t>DROGARAIA</t>
+        </is>
+      </c>
+      <c r="M54" s="18" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="N54" s="25" t="inlineStr"/>
       <c r="O54" s="24" t="inlineStr">
         <is>

</xml_diff>